<commit_message>
fixing issues and updating all of the framework
</commit_message>
<xml_diff>
--- a/src/test/resources/data/api-data.xlsx
+++ b/src/test/resources/data/api-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="60">
   <si>
     <t/>
   </si>
@@ -183,6 +183,18 @@
   </si>
   <si>
     <t>/90210</t>
+  </si>
+  <si>
+    <t>expectedCountryName</t>
+  </si>
+  <si>
+    <t>expectedAbbreviation</t>
+  </si>
+  <si>
+    <t>expectedStatus</t>
+  </si>
+  <si>
+    <t>404</t>
   </si>
 </sst>
 </file>
@@ -254,13 +266,13 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="10.15234375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="12.14453125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="11.4140625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="43.75390625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="8.59765625" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="9.2265625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="7.26953125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="10.15234375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.14453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.4140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="43.75390625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="8.59765625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="9.2265625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -408,30 +420,69 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="7.26953125"/>
+    <col min="2" max="2" width="10.15234375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="19.875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="19.1484375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="2">
         <v>1</v>
       </c>
+      <c r="B1" t="s" s="2">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s" s="2">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s" s="2">
+        <v>57</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
         <v>8</v>
       </c>
+      <c r="B2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>11</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
         <v>11</v>
       </c>
+      <c r="B3" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>11</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
         <v>39</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -444,9 +495,9 @@
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="25.56640625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="7.26953125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.15234375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="25.56640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="7.26953125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="10.15234375"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,30 +573,43 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="6.69140625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="6.69140625"/>
+    <col min="2" max="2" width="13.58203125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="4">
         <v>52</v>
       </c>
+      <c r="B1" t="s" s="4">
+        <v>58</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
         <v>53</v>
       </c>
+      <c r="B2" t="s" s="0">
+        <v>59</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
         <v>54</v>
       </c>
+      <c r="B3" t="s" s="0">
+        <v>59</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
         <v>55</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>